<commit_message>
Config: Criterio de Mes append
</commit_message>
<xml_diff>
--- a/dados/Unico_Acompanhamento_Programa_2026-20260526092151.xlsx
+++ b/dados/Unico_Acompanhamento_Programa_2026-20260526092151.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{3BFB1D67-B14B-499A-9732-AB72FC21465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35F59B22-2DA0-40D5-A35D-413E3E39D3EA}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{7BEDBE9F-36BD-4617-996F-6BA139BC564D}"/>
+    <workbookView xWindow="4800" yWindow="585" windowWidth="14355" windowHeight="9075" activeTab="1" xr2:uid="{7BEDBE9F-36BD-4617-996F-6BA139BC564D}"/>
   </bookViews>
   <sheets>
     <sheet name="Apuração" sheetId="9" r:id="rId1"/>
@@ -9515,6 +9515,45 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -9731,45 +9770,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -10529,24 +10529,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D4995A3B-399A-4C00-B9C6-DE2CF4259F41}" name="TB_APURACAO_KPIS" displayName="TB_APURACAO_KPIS" ref="B30:I34" totalsRowShown="0" headerRowDxfId="89">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D4995A3B-399A-4C00-B9C6-DE2CF4259F41}" name="TB_APURACAO_KPIS" displayName="TB_APURACAO_KPIS" ref="B30:I34" totalsRowShown="0" headerRowDxfId="74">
   <autoFilter ref="B30:I34" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5330A6FC-1100-458A-AA09-9E9F571349FC}" name="TODOS"/>
-    <tableColumn id="2" xr3:uid="{54095AC6-3B89-4408-BCA7-E30189BEA06F}" name="FAT." dataDxfId="88" dataCellStyle="Porcentagem"/>
-    <tableColumn id="3" xr3:uid="{9F2EE61B-726D-42A5-9FA5-9D132DC1D299}" name="Cob Pond" dataDxfId="87" dataCellStyle="Porcentagem"/>
-    <tableColumn id="4" xr3:uid="{EE5BA1D5-743E-4563-97A7-CB47D572F9F4}" name="Sort Pond" dataDxfId="86" dataCellStyle="Porcentagem"/>
-    <tableColumn id="5" xr3:uid="{9665DFFC-A9B5-4A30-BF26-34CEB3708EC5}" name="Exec Pond" dataDxfId="85" dataCellStyle="Porcentagem"/>
-    <tableColumn id="6" xr3:uid="{EFCAAFF5-77D6-43E5-AD9E-F01C06AB6C84}" name="Cob Num." dataDxfId="84" dataCellStyle="Porcentagem"/>
-    <tableColumn id="7" xr3:uid="{F1DE7AEB-3110-4C0C-BCB2-25033D309919}" name="Sort Num." dataDxfId="83" dataCellStyle="Porcentagem"/>
-    <tableColumn id="8" xr3:uid="{24D06F6C-9CE4-4368-B1E4-FB4F9AD825B3}" name="TT" dataDxfId="82" dataCellStyle="Porcentagem"/>
+    <tableColumn id="2" xr3:uid="{54095AC6-3B89-4408-BCA7-E30189BEA06F}" name="FAT." dataDxfId="73" dataCellStyle="Porcentagem"/>
+    <tableColumn id="3" xr3:uid="{9F2EE61B-726D-42A5-9FA5-9D132DC1D299}" name="Cob Pond" dataDxfId="72" dataCellStyle="Porcentagem"/>
+    <tableColumn id="4" xr3:uid="{EE5BA1D5-743E-4563-97A7-CB47D572F9F4}" name="Sort Pond" dataDxfId="71" dataCellStyle="Porcentagem"/>
+    <tableColumn id="5" xr3:uid="{9665DFFC-A9B5-4A30-BF26-34CEB3708EC5}" name="Exec Pond" dataDxfId="70" dataCellStyle="Porcentagem"/>
+    <tableColumn id="6" xr3:uid="{EFCAAFF5-77D6-43E5-AD9E-F01C06AB6C84}" name="Cob Num." dataDxfId="69" dataCellStyle="Porcentagem"/>
+    <tableColumn id="7" xr3:uid="{F1DE7AEB-3110-4C0C-BCB2-25033D309919}" name="Sort Num." dataDxfId="68" dataCellStyle="Porcentagem"/>
+    <tableColumn id="8" xr3:uid="{24D06F6C-9CE4-4368-B1E4-FB4F9AD825B3}" name="TT" dataDxfId="67" dataCellStyle="Porcentagem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A724E05-604A-44A5-A7E4-14CC3D185A11}" name="TB_APURACAO_VALOR_COB" displayName="TB_APURACAO_VALOR_COB" ref="B48:D52" totalsRowShown="0" headerRowDxfId="81">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A724E05-604A-44A5-A7E4-14CC3D185A11}" name="TB_APURACAO_VALOR_COB" displayName="TB_APURACAO_VALOR_COB" ref="B48:D52" totalsRowShown="0" headerRowDxfId="66">
   <autoFilter ref="B48:D52" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{967F361C-5A9B-44CE-BA60-DBCCC368C089}" name="Estado"/>
@@ -10558,7 +10558,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3538589A-C376-4F8D-97E5-D5D3AC2B41BE}" name="TB_METAS_E_REALIZADO" displayName="TB_METAS_E_REALIZADO" ref="B9:N33" totalsRowShown="0" headerRowDxfId="80" dataDxfId="79">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3538589A-C376-4F8D-97E5-D5D3AC2B41BE}" name="TB_METAS_E_REALIZADO" displayName="TB_METAS_E_REALIZADO" ref="B9:N33" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88">
   <autoFilter ref="B9:N33" xr:uid="{3538589A-C376-4F8D-97E5-D5D3AC2B41BE}">
     <filterColumn colId="3">
       <filters>
@@ -10567,19 +10567,19 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="13">
-    <tableColumn id="13" xr3:uid="{FB4C7745-A3A3-4599-B023-D4E2026DAEE8}" name="Região" dataDxfId="78"/>
-    <tableColumn id="1" xr3:uid="{1FBC83D7-82B4-4917-9CEB-27A0ED8B0D00}" name="AE" dataDxfId="77"/>
-    <tableColumn id="2" xr3:uid="{5E244AEB-29ED-471C-A8C0-C49B61F061A6}" name="KPI" dataDxfId="76"/>
-    <tableColumn id="3" xr3:uid="{3B82D024-860C-4283-94BC-782185EE9038}" name="BU" dataDxfId="75"/>
-    <tableColumn id="11" xr3:uid="{2C237177-FB9A-49BD-935F-D25E388F1AAD}" name="Unidade de Medida" dataDxfId="74"/>
-    <tableColumn id="4" xr3:uid="{86263374-3091-4ADB-B592-40FBF93E4BCC}" name="(100% do ganho)" dataDxfId="73" dataCellStyle="Vírgula"/>
-    <tableColumn id="5" xr3:uid="{AC6DF6C1-4E77-40B4-B1E1-D199723EAE20}" name="(50% do ganho)" dataDxfId="72" dataCellStyle="Vírgula"/>
-    <tableColumn id="6" xr3:uid="{115B3377-8C6A-4CAD-911C-CE0C28CD86C2}" name=" (30% do ganho)" dataDxfId="71" dataCellStyle="Vírgula"/>
-    <tableColumn id="7" xr3:uid="{48DB6C35-BA8D-45F8-B75D-187899B8AAB7}" name="Potencial Ganho" dataDxfId="70" dataCellStyle="Porcentagem"/>
-    <tableColumn id="8" xr3:uid="{204A3A88-CA1E-411E-87F3-6AD68B4C665A}" name="Realizado" dataDxfId="69" dataCellStyle="Vírgula"/>
-    <tableColumn id="12" xr3:uid="{F8B1F140-7557-42E9-9EB2-F9C84D44463C}" name="% da Meta 1" dataDxfId="68" dataCellStyle="Porcentagem"/>
-    <tableColumn id="9" xr3:uid="{C5C90530-3009-4EE8-A0BB-6CC540C29A70}" name="Faixa" dataDxfId="67"/>
-    <tableColumn id="10" xr3:uid="{ABB3BEA4-8878-4B21-A57A-117D2F42B3B4}" name="Ganho" dataDxfId="66" dataCellStyle="Porcentagem"/>
+    <tableColumn id="13" xr3:uid="{FB4C7745-A3A3-4599-B023-D4E2026DAEE8}" name="Região" dataDxfId="87"/>
+    <tableColumn id="1" xr3:uid="{1FBC83D7-82B4-4917-9CEB-27A0ED8B0D00}" name="AE" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{5E244AEB-29ED-471C-A8C0-C49B61F061A6}" name="KPI" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{3B82D024-860C-4283-94BC-782185EE9038}" name="BU" dataDxfId="84"/>
+    <tableColumn id="11" xr3:uid="{2C237177-FB9A-49BD-935F-D25E388F1AAD}" name="Unidade de Medida" dataDxfId="83"/>
+    <tableColumn id="4" xr3:uid="{86263374-3091-4ADB-B592-40FBF93E4BCC}" name="(100% do ganho)" dataDxfId="82" dataCellStyle="Vírgula"/>
+    <tableColumn id="5" xr3:uid="{AC6DF6C1-4E77-40B4-B1E1-D199723EAE20}" name="(50% do ganho)" dataDxfId="81" dataCellStyle="Vírgula"/>
+    <tableColumn id="6" xr3:uid="{115B3377-8C6A-4CAD-911C-CE0C28CD86C2}" name=" (30% do ganho)" dataDxfId="80" dataCellStyle="Vírgula"/>
+    <tableColumn id="7" xr3:uid="{48DB6C35-BA8D-45F8-B75D-187899B8AAB7}" name="Potencial Ganho" dataDxfId="79" dataCellStyle="Porcentagem"/>
+    <tableColumn id="8" xr3:uid="{204A3A88-CA1E-411E-87F3-6AD68B4C665A}" name="Realizado" dataDxfId="78" dataCellStyle="Vírgula"/>
+    <tableColumn id="12" xr3:uid="{F8B1F140-7557-42E9-9EB2-F9C84D44463C}" name="% da Meta 1" dataDxfId="77" dataCellStyle="Porcentagem"/>
+    <tableColumn id="9" xr3:uid="{C5C90530-3009-4EE8-A0BB-6CC540C29A70}" name="Faixa" dataDxfId="76"/>
+    <tableColumn id="10" xr3:uid="{ABB3BEA4-8878-4B21-A57A-117D2F42B3B4}" name="Ganho" dataDxfId="75" dataCellStyle="Porcentagem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Cofig: DataFrame principal Set
</commit_message>
<xml_diff>
--- a/dados/Unico_Acompanhamento_Programa_2026-20260526092151.xlsx
+++ b/dados/Unico_Acompanhamento_Programa_2026-20260526092151.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b234acbc490037a6/Desktop/Projetos/Uni.co/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{3BFB1D67-B14B-499A-9732-AB72FC21465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{35F59B22-2DA0-40D5-A35D-413E3E39D3EA}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{3BFB1D67-B14B-499A-9732-AB72FC21465C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1CF2696-3436-4A9C-948C-1872A7933138}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="585" windowWidth="14355" windowHeight="9075" activeTab="1" xr2:uid="{7BEDBE9F-36BD-4617-996F-6BA139BC564D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="6" xr2:uid="{7BEDBE9F-36BD-4617-996F-6BA139BC564D}"/>
   </bookViews>
   <sheets>
     <sheet name="Apuração" sheetId="9" r:id="rId1"/>
@@ -8993,157 +8993,6 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color theme="0"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF0042E7"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="hair">
-          <color auto="1"/>
-        </left>
-        <right style="hair">
-          <color auto="1"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-      <protection locked="0" hidden="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="minor"/>
@@ -9515,45 +9364,6 @@
       <protection locked="0" hidden="0"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="14" formatCode="0.00%"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="4" tint="-0.249977111117893"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -9770,6 +9580,196 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="14" formatCode="0.00%"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF0042E7"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="hair">
+          <color auto="1"/>
+        </left>
+        <right style="hair">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+      <protection locked="0" hidden="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -10529,24 +10529,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D4995A3B-399A-4C00-B9C6-DE2CF4259F41}" name="TB_APURACAO_KPIS" displayName="TB_APURACAO_KPIS" ref="B30:I34" totalsRowShown="0" headerRowDxfId="74">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D4995A3B-399A-4C00-B9C6-DE2CF4259F41}" name="TB_APURACAO_KPIS" displayName="TB_APURACAO_KPIS" ref="B30:I34" totalsRowShown="0" headerRowDxfId="80">
   <autoFilter ref="B30:I34" xr:uid="{00000000-0009-0000-0100-000005000000}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{5330A6FC-1100-458A-AA09-9E9F571349FC}" name="TODOS"/>
-    <tableColumn id="2" xr3:uid="{54095AC6-3B89-4408-BCA7-E30189BEA06F}" name="FAT." dataDxfId="73" dataCellStyle="Porcentagem"/>
-    <tableColumn id="3" xr3:uid="{9F2EE61B-726D-42A5-9FA5-9D132DC1D299}" name="Cob Pond" dataDxfId="72" dataCellStyle="Porcentagem"/>
-    <tableColumn id="4" xr3:uid="{EE5BA1D5-743E-4563-97A7-CB47D572F9F4}" name="Sort Pond" dataDxfId="71" dataCellStyle="Porcentagem"/>
-    <tableColumn id="5" xr3:uid="{9665DFFC-A9B5-4A30-BF26-34CEB3708EC5}" name="Exec Pond" dataDxfId="70" dataCellStyle="Porcentagem"/>
-    <tableColumn id="6" xr3:uid="{EFCAAFF5-77D6-43E5-AD9E-F01C06AB6C84}" name="Cob Num." dataDxfId="69" dataCellStyle="Porcentagem"/>
-    <tableColumn id="7" xr3:uid="{F1DE7AEB-3110-4C0C-BCB2-25033D309919}" name="Sort Num." dataDxfId="68" dataCellStyle="Porcentagem"/>
-    <tableColumn id="8" xr3:uid="{24D06F6C-9CE4-4368-B1E4-FB4F9AD825B3}" name="TT" dataDxfId="67" dataCellStyle="Porcentagem"/>
+    <tableColumn id="2" xr3:uid="{54095AC6-3B89-4408-BCA7-E30189BEA06F}" name="FAT." dataDxfId="79" dataCellStyle="Porcentagem"/>
+    <tableColumn id="3" xr3:uid="{9F2EE61B-726D-42A5-9FA5-9D132DC1D299}" name="Cob Pond" dataDxfId="78" dataCellStyle="Porcentagem"/>
+    <tableColumn id="4" xr3:uid="{EE5BA1D5-743E-4563-97A7-CB47D572F9F4}" name="Sort Pond" dataDxfId="77" dataCellStyle="Porcentagem"/>
+    <tableColumn id="5" xr3:uid="{9665DFFC-A9B5-4A30-BF26-34CEB3708EC5}" name="Exec Pond" dataDxfId="76" dataCellStyle="Porcentagem"/>
+    <tableColumn id="6" xr3:uid="{EFCAAFF5-77D6-43E5-AD9E-F01C06AB6C84}" name="Cob Num." dataDxfId="75" dataCellStyle="Porcentagem"/>
+    <tableColumn id="7" xr3:uid="{F1DE7AEB-3110-4C0C-BCB2-25033D309919}" name="Sort Num." dataDxfId="74" dataCellStyle="Porcentagem"/>
+    <tableColumn id="8" xr3:uid="{24D06F6C-9CE4-4368-B1E4-FB4F9AD825B3}" name="TT" dataDxfId="73" dataCellStyle="Porcentagem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A724E05-604A-44A5-A7E4-14CC3D185A11}" name="TB_APURACAO_VALOR_COB" displayName="TB_APURACAO_VALOR_COB" ref="B48:D52" totalsRowShown="0" headerRowDxfId="66">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1A724E05-604A-44A5-A7E4-14CC3D185A11}" name="TB_APURACAO_VALOR_COB" displayName="TB_APURACAO_VALOR_COB" ref="B48:D52" totalsRowShown="0" headerRowDxfId="72">
   <autoFilter ref="B48:D52" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{967F361C-5A9B-44CE-BA60-DBCCC368C089}" name="Estado"/>
@@ -10558,7 +10558,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3538589A-C376-4F8D-97E5-D5D3AC2B41BE}" name="TB_METAS_E_REALIZADO" displayName="TB_METAS_E_REALIZADO" ref="B9:N33" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{3538589A-C376-4F8D-97E5-D5D3AC2B41BE}" name="TB_METAS_E_REALIZADO" displayName="TB_METAS_E_REALIZADO" ref="B9:N33" totalsRowShown="0" headerRowDxfId="71" dataDxfId="70">
   <autoFilter ref="B9:N33" xr:uid="{3538589A-C376-4F8D-97E5-D5D3AC2B41BE}">
     <filterColumn colId="3">
       <filters>
@@ -10567,71 +10567,71 @@
     </filterColumn>
   </autoFilter>
   <tableColumns count="13">
-    <tableColumn id="13" xr3:uid="{FB4C7745-A3A3-4599-B023-D4E2026DAEE8}" name="Região" dataDxfId="87"/>
-    <tableColumn id="1" xr3:uid="{1FBC83D7-82B4-4917-9CEB-27A0ED8B0D00}" name="AE" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{5E244AEB-29ED-471C-A8C0-C49B61F061A6}" name="KPI" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{3B82D024-860C-4283-94BC-782185EE9038}" name="BU" dataDxfId="84"/>
-    <tableColumn id="11" xr3:uid="{2C237177-FB9A-49BD-935F-D25E388F1AAD}" name="Unidade de Medida" dataDxfId="83"/>
-    <tableColumn id="4" xr3:uid="{86263374-3091-4ADB-B592-40FBF93E4BCC}" name="(100% do ganho)" dataDxfId="82" dataCellStyle="Vírgula"/>
-    <tableColumn id="5" xr3:uid="{AC6DF6C1-4E77-40B4-B1E1-D199723EAE20}" name="(50% do ganho)" dataDxfId="81" dataCellStyle="Vírgula"/>
-    <tableColumn id="6" xr3:uid="{115B3377-8C6A-4CAD-911C-CE0C28CD86C2}" name=" (30% do ganho)" dataDxfId="80" dataCellStyle="Vírgula"/>
-    <tableColumn id="7" xr3:uid="{48DB6C35-BA8D-45F8-B75D-187899B8AAB7}" name="Potencial Ganho" dataDxfId="79" dataCellStyle="Porcentagem"/>
-    <tableColumn id="8" xr3:uid="{204A3A88-CA1E-411E-87F3-6AD68B4C665A}" name="Realizado" dataDxfId="78" dataCellStyle="Vírgula"/>
-    <tableColumn id="12" xr3:uid="{F8B1F140-7557-42E9-9EB2-F9C84D44463C}" name="% da Meta 1" dataDxfId="77" dataCellStyle="Porcentagem"/>
-    <tableColumn id="9" xr3:uid="{C5C90530-3009-4EE8-A0BB-6CC540C29A70}" name="Faixa" dataDxfId="76"/>
-    <tableColumn id="10" xr3:uid="{ABB3BEA4-8878-4B21-A57A-117D2F42B3B4}" name="Ganho" dataDxfId="75" dataCellStyle="Porcentagem"/>
+    <tableColumn id="13" xr3:uid="{FB4C7745-A3A3-4599-B023-D4E2026DAEE8}" name="Região" dataDxfId="69"/>
+    <tableColumn id="1" xr3:uid="{1FBC83D7-82B4-4917-9CEB-27A0ED8B0D00}" name="AE" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{5E244AEB-29ED-471C-A8C0-C49B61F061A6}" name="KPI" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{3B82D024-860C-4283-94BC-782185EE9038}" name="BU" dataDxfId="66"/>
+    <tableColumn id="11" xr3:uid="{2C237177-FB9A-49BD-935F-D25E388F1AAD}" name="Unidade de Medida" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{86263374-3091-4ADB-B592-40FBF93E4BCC}" name="(100% do ganho)" dataDxfId="64" dataCellStyle="Vírgula"/>
+    <tableColumn id="5" xr3:uid="{AC6DF6C1-4E77-40B4-B1E1-D199723EAE20}" name="(50% do ganho)" dataDxfId="63" dataCellStyle="Vírgula"/>
+    <tableColumn id="6" xr3:uid="{115B3377-8C6A-4CAD-911C-CE0C28CD86C2}" name=" (30% do ganho)" dataDxfId="62" dataCellStyle="Vírgula"/>
+    <tableColumn id="7" xr3:uid="{48DB6C35-BA8D-45F8-B75D-187899B8AAB7}" name="Potencial Ganho" dataDxfId="61" dataCellStyle="Porcentagem"/>
+    <tableColumn id="8" xr3:uid="{204A3A88-CA1E-411E-87F3-6AD68B4C665A}" name="Realizado" dataDxfId="60" dataCellStyle="Vírgula"/>
+    <tableColumn id="12" xr3:uid="{F8B1F140-7557-42E9-9EB2-F9C84D44463C}" name="% da Meta 1" dataDxfId="59" dataCellStyle="Porcentagem"/>
+    <tableColumn id="9" xr3:uid="{C5C90530-3009-4EE8-A0BB-6CC540C29A70}" name="Faixa" dataDxfId="58"/>
+    <tableColumn id="10" xr3:uid="{ABB3BEA4-8878-4B21-A57A-117D2F42B3B4}" name="Ganho" dataDxfId="57" dataCellStyle="Porcentagem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6AF76526-113C-4232-9C7F-ED21D262E981}" name="TB_SORTIMENTO_POND" displayName="TB_SORTIMENTO_POND" ref="B8:K320" totalsRowShown="0" headerRowDxfId="65" dataDxfId="64">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6AF76526-113C-4232-9C7F-ED21D262E981}" name="TB_SORTIMENTO_POND" displayName="TB_SORTIMENTO_POND" ref="B8:K320" totalsRowShown="0" headerRowDxfId="56" dataDxfId="55">
   <autoFilter ref="B8:K320" xr:uid="{6AF76526-113C-4232-9C7F-ED21D262E981}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{70462B59-80DF-47F8-85D2-4C0EED5CBA92}" name="Região do Sortimento" dataDxfId="63"/>
-    <tableColumn id="2" xr3:uid="{0581EADB-E1D8-4D4E-AB1F-ABCF66C6251A}" name="AE" dataDxfId="62"/>
-    <tableColumn id="3" xr3:uid="{AB652728-0371-4E9E-BD35-635796DB6706}" name="BU" dataDxfId="61"/>
-    <tableColumn id="4" xr3:uid="{B812C714-D502-4F4C-81F2-1ED7917A6DB4}" name="Categoria" dataDxfId="60"/>
-    <tableColumn id="5" xr3:uid="{BFCBCFB7-E329-4C9C-BB74-C29505AFEFD3}" name="Descricao" dataDxfId="59"/>
-    <tableColumn id="6" xr3:uid="{9A678B47-CE8D-4B34-8C0B-AA45CC0D7372}" name="EAN Regular" dataDxfId="58"/>
-    <tableColumn id="7" xr3:uid="{20C660B7-A423-4EA8-9D57-51C188EA5796}" name="Outros EANS válidos" dataDxfId="57"/>
-    <tableColumn id="10" xr3:uid="{610B1D60-4A29-4D4A-B187-CD0DD9DFD8AB}" name="Total de Redes" dataDxfId="56"/>
-    <tableColumn id="8" xr3:uid="{DBBC44BA-00D7-41A2-94B7-7F8EE7295D19}" name="Redes com Compra no mês" dataDxfId="55"/>
-    <tableColumn id="9" xr3:uid="{0DAF926D-EBFC-47D3-BFA6-0965BE18D7B1}" name="% das Redes" dataDxfId="54" dataCellStyle="Porcentagem"/>
+    <tableColumn id="1" xr3:uid="{70462B59-80DF-47F8-85D2-4C0EED5CBA92}" name="Região do Sortimento" dataDxfId="54"/>
+    <tableColumn id="2" xr3:uid="{0581EADB-E1D8-4D4E-AB1F-ABCF66C6251A}" name="AE" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{AB652728-0371-4E9E-BD35-635796DB6706}" name="BU" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{B812C714-D502-4F4C-81F2-1ED7917A6DB4}" name="Categoria" dataDxfId="51"/>
+    <tableColumn id="5" xr3:uid="{BFCBCFB7-E329-4C9C-BB74-C29505AFEFD3}" name="Descricao" dataDxfId="50"/>
+    <tableColumn id="6" xr3:uid="{9A678B47-CE8D-4B34-8C0B-AA45CC0D7372}" name="EAN Regular" dataDxfId="49"/>
+    <tableColumn id="7" xr3:uid="{20C660B7-A423-4EA8-9D57-51C188EA5796}" name="Outros EANS válidos" dataDxfId="48"/>
+    <tableColumn id="10" xr3:uid="{610B1D60-4A29-4D4A-B187-CD0DD9DFD8AB}" name="Total de Redes" dataDxfId="47"/>
+    <tableColumn id="8" xr3:uid="{DBBC44BA-00D7-41A2-94B7-7F8EE7295D19}" name="Redes com Compra no mês" dataDxfId="46"/>
+    <tableColumn id="9" xr3:uid="{0DAF926D-EBFC-47D3-BFA6-0965BE18D7B1}" name="% das Redes" dataDxfId="45" dataCellStyle="Porcentagem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{89653739-F875-4D30-A6D4-143F605A695B}" name="TB_SORTIMENTO_NUM" displayName="TB_SORTIMENTO_NUM" ref="B8:I85" totalsRowShown="0" headerRowDxfId="53" dataDxfId="52">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{89653739-F875-4D30-A6D4-143F605A695B}" name="TB_SORTIMENTO_NUM" displayName="TB_SORTIMENTO_NUM" ref="B8:I85" totalsRowShown="0" headerRowDxfId="44" dataDxfId="43">
   <autoFilter ref="B8:I85" xr:uid="{89653739-F875-4D30-A6D4-143F605A695B}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{F012D9F9-4AA9-4DD8-8D2C-386F463D46BD}" name="Região do Sortimento" dataDxfId="51"/>
-    <tableColumn id="2" xr3:uid="{C930A51D-467F-4F88-99D7-DC0DAF4C88DC}" name="AE" dataDxfId="50"/>
-    <tableColumn id="3" xr3:uid="{2172EEA3-6E07-439C-9317-D4BC4CD2DB72}" name="BU" dataDxfId="49"/>
-    <tableColumn id="4" xr3:uid="{E392C421-19F5-455C-BB4E-F901EBE62E4D}" name="Categoria" dataDxfId="48"/>
-    <tableColumn id="5" xr3:uid="{0E460137-2D05-4B06-ACE2-BE9A10A7F8EB}" name="PPA" dataDxfId="47"/>
-    <tableColumn id="8" xr3:uid="{09F3908B-349C-408C-BD3B-111223AC241F}" name="Qtde de Lojas da Numérica A e B" dataDxfId="46"/>
-    <tableColumn id="6" xr3:uid="{D35D2950-2C90-4B51-8B9F-9F281297DAD7}" name="Qtde de Lojas da Numérica A e B com compra do PPA no bimestre móvel" dataDxfId="45"/>
-    <tableColumn id="7" xr3:uid="{88E10F0B-E51E-4A14-9392-78DBAECBE14A}" name="% das Lojas da Numérica A e B com compra do PPA no bimestre móvel" dataDxfId="44" dataCellStyle="Porcentagem"/>
+    <tableColumn id="1" xr3:uid="{F012D9F9-4AA9-4DD8-8D2C-386F463D46BD}" name="Região do Sortimento" dataDxfId="42"/>
+    <tableColumn id="2" xr3:uid="{C930A51D-467F-4F88-99D7-DC0DAF4C88DC}" name="AE" dataDxfId="41"/>
+    <tableColumn id="3" xr3:uid="{2172EEA3-6E07-439C-9317-D4BC4CD2DB72}" name="BU" dataDxfId="40"/>
+    <tableColumn id="4" xr3:uid="{E392C421-19F5-455C-BB4E-F901EBE62E4D}" name="Categoria" dataDxfId="39"/>
+    <tableColumn id="5" xr3:uid="{0E460137-2D05-4B06-ACE2-BE9A10A7F8EB}" name="PPA" dataDxfId="38"/>
+    <tableColumn id="8" xr3:uid="{09F3908B-349C-408C-BD3B-111223AC241F}" name="Qtde de Lojas da Numérica A e B" dataDxfId="37"/>
+    <tableColumn id="6" xr3:uid="{D35D2950-2C90-4B51-8B9F-9F281297DAD7}" name="Qtde de Lojas da Numérica A e B com compra do PPA no bimestre móvel" dataDxfId="36"/>
+    <tableColumn id="7" xr3:uid="{88E10F0B-E51E-4A14-9392-78DBAECBE14A}" name="% das Lojas da Numérica A e B com compra do PPA no bimestre móvel" dataDxfId="35" dataCellStyle="Porcentagem"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{12A47C04-14E2-46CF-A2C3-37D7752CFC50}" name="TB_EANS_PPA" displayName="TB_EANS_PPA" ref="B8:H934" totalsRowShown="0" headerRowDxfId="43" dataDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{12A47C04-14E2-46CF-A2C3-37D7752CFC50}" name="TB_EANS_PPA" displayName="TB_EANS_PPA" ref="B8:H934" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88">
   <autoFilter ref="B8:H934" xr:uid="{12A47C04-14E2-46CF-A2C3-37D7752CFC50}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{EA0D1BC5-0C18-4157-92A9-CCCBDF42516D}" name="Região do Sortimento" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{F77A144A-8119-460F-ADF0-928B6A88BB30}" name="AE" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{D1AD7BA7-0288-4906-8914-B01801D72609}" name="BU" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{5C5C0594-8D3E-4AAA-BF64-C6A5C37F990F}" name="Categoria" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{004D5BE0-7D5A-472C-9294-8455DF372558}" name="PPA" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{B0A59FAE-56CE-4E50-94C5-291E32EB73ED}" name="Descrição" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{CC413941-E897-43BE-B4DC-8432EA5C62DE}" name="EAN Regular " dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{EA0D1BC5-0C18-4157-92A9-CCCBDF42516D}" name="Região do Sortimento" dataDxfId="87"/>
+    <tableColumn id="2" xr3:uid="{F77A144A-8119-460F-ADF0-928B6A88BB30}" name="AE" dataDxfId="86"/>
+    <tableColumn id="3" xr3:uid="{D1AD7BA7-0288-4906-8914-B01801D72609}" name="BU" dataDxfId="85"/>
+    <tableColumn id="4" xr3:uid="{5C5C0594-8D3E-4AAA-BF64-C6A5C37F990F}" name="Categoria" dataDxfId="84"/>
+    <tableColumn id="5" xr3:uid="{004D5BE0-7D5A-472C-9294-8455DF372558}" name="PPA" dataDxfId="83"/>
+    <tableColumn id="6" xr3:uid="{B0A59FAE-56CE-4E50-94C5-291E32EB73ED}" name="Descrição" dataDxfId="82"/>
+    <tableColumn id="7" xr3:uid="{CC413941-E897-43BE-B4DC-8432EA5C62DE}" name="EAN Regular " dataDxfId="81"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>